<commit_message>
Corriger les chemins subSection obsoletes dans le mapping ExposureInformation f7065029d8b040b6d3a2c13e23ba7cb02315d43c
</commit_message>
<xml_diff>
--- a/fix-target-codes-and-display/ig/FRSectionExposureInformationLMCDAFHIR.xlsx
+++ b/fix-target-codes-and-display/ig/FRSectionExposureInformationLMCDAFHIR.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="56">
   <si>
     <t>Property</t>
   </si>
@@ -61,7 +61,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-25T11:34:21+00:00</t>
+    <t>2026-08-25T11:56:50+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -145,13 +145,13 @@
     <t>Section.text</t>
   </si>
   <si>
-    <t>FRLMExposureInformation.subSection.quantityExposure</t>
+    <t>FRLMExposureInformation.entry.quantityExposure</t>
   </si>
   <si>
     <t>Section.entry:frDicomQuantite.observation</t>
   </si>
   <si>
-    <t>FRLMExposureInformation.subSection.radiopharmaceuticalAdministration</t>
+    <t>FRLMExposureInformation.entry.radiopharmaceuticalAdministration</t>
   </si>
   <si>
     <t>Section.entry:frDicomAdministrationRadiopharmaceutique.substanceAdministration</t>
@@ -175,16 +175,10 @@
     <t>Composition.section.text</t>
   </si>
   <si>
-    <t>FRLMExposureInformation.entry.quantityExposure</t>
-  </si>
-  <si>
     <t>Composition.section.entry</t>
   </si>
   <si>
     <t>FRObservationRadiationExposureDocument</t>
-  </si>
-  <si>
-    <t>FRLMExposureInformation.entry.radiopharmaceuticalAdministration</t>
   </si>
   <si>
     <t>FRMedicationAdministrationDocument</t>
@@ -660,32 +654,32 @@
     </row>
     <row r="7">
       <c r="A7" t="s" s="2">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D7" t="s" s="2">
+        <v>53</v>
+      </c>
+      <c r="E7" t="s" s="2">
         <v>54</v>
-      </c>
-      <c r="E7" t="s" s="2">
-        <v>55</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="2">
-        <v>56</v>
+        <v>45</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D8" t="s" s="2">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E8" t="s" s="2">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>

</xml_diff>